<commit_message>
Redesign the portfolio: playable island town hero, bold playful theme, day/night mode
- Home page hero is an isometric SVG town where each building links to a project,
  with tree planting, an explore counter and a delivery truck on the road
- New shared theme (style.css, site.js): chunky cards, hover motion, scroll reveals,
  day/night toggle, confetti on copy, reduced-motion support
- Project pages pick up the theme with a colour per project
- Discrepancy Checker page leads with results; formulas collapsed; public workbook
  drops the study guide and practice wording
</commit_message>
<xml_diff>
--- a/demos/discrepancy-checker/Discrepancy_Checker_Sample.xlsx
+++ b/demos/discrepancy-checker/Discrepancy_Checker_Sample.xlsx
@@ -14,7 +14,6 @@
     <sheet name="Billing" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Items" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Lists" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Formula Guide" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="ReasonCodes">Lists!$A$2:$A$8</definedName>
@@ -40,7 +39,7 @@
     <numFmt numFmtId="169" formatCode="mmm yyyy"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -152,17 +151,6 @@
       <color rgb="001F3A5F"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F3A5F"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Courier New"/>
-      <color rgb="001F2933"/>
-      <sz val="9"/>
-    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -262,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -354,19 +342,6 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1173,7 +1148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C31"/>
+  <dimension ref="B2:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1198,7 +1173,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Practice workbook. Every company, SKU, quantity, rate and dollar amount in this file is made up. Carrier names are real Canadian carriers, used only to make the receiving log look realistic.</t>
+          <t>Sample data. Every company, SKU, quantity, rate and dollar amount in this file is made up. Carrier names are real Canadian carriers, used only to make the receiving log look realistic.</t>
         </is>
       </c>
     </row>
@@ -1295,149 +1270,101 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Formula Guide</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Every formula in the file, in plain words, with the XLOOKUP version and how to build the pivot.</t>
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Colour key</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Colour key</t>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>1,250</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Blue text: typed-in values. Change these.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>1,250</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Blue text: typed-in values. Change these.</t>
+          <t>Grey cell: formula. Do not type over it.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>1,250</t>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Check</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Grey cell: formula. Do not type over it.</t>
+          <t>Red: needs a look (variance, mismatch or billing difference).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Red: needs a look (variance, mismatch or billing difference).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
           <t>Green text: matches.</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>How to use it</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>How to use it</t>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Enter physical counts in Inventory column D and give every Check row a reason code.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Step 1</t>
+          <t>Step 2</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Type the physical count in Inventory column D. Variance, status and dollar impact update by themselves.</t>
+          <t>Log receipts in Receiving and storage invoices in Billing. Rates and the tolerance live on Lists.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 3</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>For every row marked Check, pick a reason from the dropdown in column J.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Log each receipt in Receiving: PO qty, packing slip qty and what was actually received.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Step 4</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Enter each storage invoice in Billing. The expected amount comes from the client's rate in Lists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
           <t>To add rows, copy the last row down so the grey formula cells come with it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Read the Dashboard. Filters on each sheet (header arrows) show only the rows marked Check.</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1380,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -8336,605 +8262,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00B9770E"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B2:F32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="B2" s="45" t="inlineStr">
-        <is>
-          <t>Formula Guide</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Every formula in the workbook, what it does, and the XLOOKUP version where one applies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="46" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="C5" s="46" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D5" s="46" t="inlineStr">
-        <is>
-          <t>Formula</t>
-        </is>
-      </c>
-      <c r="E5" s="46" t="inlineStr">
-        <is>
-          <t>What it does</t>
-        </is>
-      </c>
-      <c r="F5" s="46" t="inlineStr">
-        <is>
-          <t>XLOOKUP version (Excel 365)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="B6" s="47" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C6" s="47" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D6" s="48" t="inlineStr">
-        <is>
-          <t>=IFERROR(INDEX(Items!$B$2:$B$200,MATCH($A2,Items!$A$2:$A$200,0)),"SKU not found")</t>
-        </is>
-      </c>
-      <c r="E6" s="47" t="inlineStr">
-        <is>
-          <t>MATCH finds which row of the Items list holds this SKU (0 means exact match). INDEX returns the description from that same row. IFERROR shows a message instead of an error when the SKU is not in the list.</t>
-        </is>
-      </c>
-      <c r="F6" s="48" t="inlineStr">
-        <is>
-          <t>=XLOOKUP($A2,Items!$A$2:$A$200,Items!$B$2:$B$200,"SKU not found")</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="B7" s="47" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C7" s="47" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D7" s="48" t="inlineStr">
-        <is>
-          <t>=D2-C2</t>
-        </is>
-      </c>
-      <c r="E7" s="47" t="inlineStr">
-        <is>
-          <t>Physical count minus system qty. Negative means fewer on the shelf than the system thinks (shrink). Positive means more.</t>
-        </is>
-      </c>
-      <c r="F7" s="49" t="inlineStr"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="47" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C8" s="47" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D8" s="48" t="inlineStr">
-        <is>
-          <t>=IF(E2=0,"OK","Check")</t>
-        </is>
-      </c>
-      <c r="E8" s="47" t="inlineStr">
-        <is>
-          <t>If the variance is zero the row is OK, otherwise it needs a look. Conditional formatting turns Check red.</t>
-        </is>
-      </c>
-      <c r="F8" s="49" t="inlineStr"/>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="B9" s="47" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C9" s="47" t="inlineStr">
-        <is>
-          <t>G, H</t>
-        </is>
-      </c>
-      <c r="D9" s="49" t="inlineStr">
-        <is>
-          <t>Same INDEX/MATCH as column B</t>
-        </is>
-      </c>
-      <c r="E9" s="47" t="inlineStr">
-        <is>
-          <t>Pull the bin location and unit cost from Items. Unit cost returns 0 if the SKU is missing so the dollar maths still works.</t>
-        </is>
-      </c>
-      <c r="F9" s="48" t="inlineStr">
-        <is>
-          <t>=XLOOKUP($A2,Items!$A$2:$A$200,Items!$E$2:$E$200,0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="47" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C10" s="47" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D10" s="48" t="inlineStr">
-        <is>
-          <t>=E2*H2</t>
-        </is>
-      </c>
-      <c r="E10" s="47" t="inlineStr">
-        <is>
-          <t>Dollar impact of the variance: units off times unit cost.</t>
-        </is>
-      </c>
-      <c r="F10" s="49" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="47" t="inlineStr">
-        <is>
-          <t>Receiving</t>
-        </is>
-      </c>
-      <c r="C11" s="47" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D11" s="49" t="inlineStr">
-        <is>
-          <t>Same INDEX/MATCH as Inventory B</t>
-        </is>
-      </c>
-      <c r="E11" s="47" t="inlineStr">
-        <is>
-          <t>Description of the SKU received.</t>
-        </is>
-      </c>
-      <c r="F11" s="49" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="47" t="inlineStr">
-        <is>
-          <t>Receiving</t>
-        </is>
-      </c>
-      <c r="C12" s="47" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="D12" s="48" t="inlineStr">
-        <is>
-          <t>=I2-H2</t>
-        </is>
-      </c>
-      <c r="E12" s="47" t="inlineStr">
-        <is>
-          <t>Qty received minus packing slip qty. Negative: short shipped. Positive: over.</t>
-        </is>
-      </c>
-      <c r="F12" s="49" t="inlineStr"/>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="B13" s="47" t="inlineStr">
-        <is>
-          <t>Receiving</t>
-        </is>
-      </c>
-      <c r="C13" s="47" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="D13" s="48" t="inlineStr">
-        <is>
-          <t>=IF(J2&lt;0,"Short",IF(J2&gt;0,"Over",IF(H2&lt;&gt;G2,"PO mismatch","OK")))</t>
-        </is>
-      </c>
-      <c r="E13" s="47" t="inlineStr">
-        <is>
-          <t>Nested IF, read left to right: short first, then over. If the counts match the slip, it still checks the slip against the PO, because a supplier can ship (and bill) a different quantity than was ordered.</t>
-        </is>
-      </c>
-      <c r="F13" s="49" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="47" t="inlineStr">
-        <is>
-          <t>Receiving</t>
-        </is>
-      </c>
-      <c r="C14" s="47" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D14" s="48" t="inlineStr">
-        <is>
-          <t>="Wk "&amp;TEXT(WEEKNUM(A2,2),"00")</t>
-        </is>
-      </c>
-      <c r="E14" s="47" t="inlineStr">
-        <is>
-          <t>Week number of the receipt date, weeks starting Monday, as text like Wk 37. Used to group by week in a pivot table.</t>
-        </is>
-      </c>
-      <c r="F14" s="49" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="47" t="inlineStr">
-        <is>
-          <t>Billing</t>
-        </is>
-      </c>
-      <c r="C15" s="47" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D15" s="48" t="inlineStr">
-        <is>
-          <t>=IFERROR(INDEX(Lists!$F$2:$F$20,MATCH(B2,Lists!$E$2:$E$20,0)),0)</t>
-        </is>
-      </c>
-      <c r="E15" s="47" t="inlineStr">
-        <is>
-          <t>Looks up the client's storage rate on the Lists sheet, so a rate change is made in one place.</t>
-        </is>
-      </c>
-      <c r="F15" s="48" t="inlineStr">
-        <is>
-          <t>=XLOOKUP(B2,Lists!$E$2:$E$20,Lists!$F$2:$F$20,0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="47" t="inlineStr">
-        <is>
-          <t>Billing</t>
-        </is>
-      </c>
-      <c r="C16" s="47" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D16" s="48" t="inlineStr">
-        <is>
-          <t>=C2*D2</t>
-        </is>
-      </c>
-      <c r="E16" s="47" t="inlineStr">
-        <is>
-          <t>Expected invoice: pallets stored times rate.</t>
-        </is>
-      </c>
-      <c r="F16" s="49" t="inlineStr"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="B17" s="47" t="inlineStr">
-        <is>
-          <t>Billing</t>
-        </is>
-      </c>
-      <c r="C17" s="47" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="D17" s="48" t="inlineStr">
-        <is>
-          <t>=E2-F2</t>
-        </is>
-      </c>
-      <c r="E17" s="47" t="inlineStr">
-        <is>
-          <t>Invoiced minus expected. Positive: client overbilled. Negative: we underbilled.</t>
-        </is>
-      </c>
-      <c r="F17" s="49" t="inlineStr"/>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="B18" s="47" t="inlineStr">
-        <is>
-          <t>Billing</t>
-        </is>
-      </c>
-      <c r="C18" s="47" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D18" s="48" t="inlineStr">
-        <is>
-          <t>=IF(ABS(G2)&gt;Lists!$I$2,"Check","OK")</t>
-        </is>
-      </c>
-      <c r="E18" s="47" t="inlineStr">
-        <is>
-          <t>ABS ignores the sign, so overbilling and underbilling are both caught. The tolerance ($1.00) is one cell on Lists, so rounding cents are not flagged.</t>
-        </is>
-      </c>
-      <c r="F18" s="49" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="B19" s="47" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C19" s="47" t="inlineStr">
-        <is>
-          <t>Cards</t>
-        </is>
-      </c>
-      <c r="D19" s="48" t="inlineStr">
-        <is>
-          <t>=COUNTA(Inventory!$A$2:$A$500)</t>
-        </is>
-      </c>
-      <c r="E19" s="47" t="inlineStr">
-        <is>
-          <t>Counts non-empty cells: how many SKUs were counted. The range goes to row 500 so new rows are included.</t>
-        </is>
-      </c>
-      <c r="F19" s="49" t="inlineStr"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="47" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C20" s="47" t="inlineStr">
-        <is>
-          <t>Cards</t>
-        </is>
-      </c>
-      <c r="D20" s="48" t="inlineStr">
-        <is>
-          <t>=COUNTIF(Inventory!$F$2:$F$500,"Check")</t>
-        </is>
-      </c>
-      <c r="E20" s="47" t="inlineStr">
-        <is>
-          <t>Counts the rows whose status is Check.</t>
-        </is>
-      </c>
-      <c r="F20" s="49" t="inlineStr"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="47" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C21" s="47" t="inlineStr">
-        <is>
-          <t>Cards</t>
-        </is>
-      </c>
-      <c r="D21" s="48" t="inlineStr">
-        <is>
-          <t>=IF(B7=0,0,1-E7/B7)</t>
-        </is>
-      </c>
-      <c r="E21" s="47" t="inlineStr">
-        <is>
-          <t>Inventory accuracy: share of SKUs with no variance. The IF avoids dividing by zero on an empty sheet.</t>
-        </is>
-      </c>
-      <c r="F21" s="49" t="inlineStr"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="47" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C22" s="47" t="inlineStr">
-        <is>
-          <t>Cards</t>
-        </is>
-      </c>
-      <c r="D22" s="48" t="inlineStr">
-        <is>
-          <t>=SUMIF(Billing!$H$2:$H$500,"Check",Billing!$G$2:$G$500)</t>
-        </is>
-      </c>
-      <c r="E22" s="47" t="inlineStr">
-        <is>
-          <t>Adds the variance only for invoices flagged Check: the dollar amount that needs to be credited or rebilled.</t>
-        </is>
-      </c>
-      <c r="F22" s="49" t="inlineStr"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="47" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C23" s="47" t="inlineStr">
-        <is>
-          <t>Tables</t>
-        </is>
-      </c>
-      <c r="D23" s="48" t="inlineStr">
-        <is>
-          <t>=SUMIF(Billing!$B$2:$B$500,B51,Billing!$G$2:$G$500)</t>
-        </is>
-      </c>
-      <c r="E23" s="47" t="inlineStr">
-        <is>
-          <t>Total billing variance for the client named in column B. Same idea as COUNTIF, but adds instead of counts.</t>
-        </is>
-      </c>
-      <c r="F23" s="49" t="inlineStr"/>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="B24" s="47" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="C24" s="47" t="inlineStr">
-        <is>
-          <t>$ signs</t>
-        </is>
-      </c>
-      <c r="D24" s="49" t="inlineStr">
-        <is>
-          <t>$A$2 vs A2</t>
-        </is>
-      </c>
-      <c r="E24" s="47" t="inlineStr">
-        <is>
-          <t>A $ locks the column or row when the formula is copied. Lookup ranges are locked ($) so they do not shift; the row being checked (A2) is not, so it moves down.</t>
-        </is>
-      </c>
-      <c r="F24" s="49" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Practice: build a pivot table by SKU and by week</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>Step 1</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Click any cell in the Receiving table, then Insert &gt; PivotTable &gt; New Worksheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Drag SKU to Rows, Variance to Values (Sum). Sort ascending: the most short-shipped SKUs come first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Drag Flag to Filters and pick Short to see only short shipments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Step 4</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Swap SKU for Week in Rows to see which weeks had the most receiving problems.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Do the same on Inventory: Reason to Rows, Variance ($) to Values. That is the shrink by cause.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>After changing data, right-click the pivot &gt; Refresh. Pivots do not update on their own.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C28:F28"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>